<commit_message>
feat: agregar Growatt MAX 100KTL3, Huawei SUN2000-100KTL-M1, Sungrow SG110CX al catálogo Excel de inversores (1500V/granja)
</commit_message>
<xml_diff>
--- a/bipv_python/datos/inversores_catalogo.xlsx
+++ b/bipv_python/datos/inversores_catalogo.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo_Inversores" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo_Baterias" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Catalogo_Inversores" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Catalogo_Baterias" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:N108"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -5669,6 +5669,147 @@
       </c>
       <c r="N105" t="n">
         <v>6000</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Growatt MAX 100KTL3 LV</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>Ficha técnica oficial — sistema 1500V granja FV</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F106" t="n">
+        <v>200</v>
+      </c>
+      <c r="G106" t="n">
+        <v>200</v>
+      </c>
+      <c r="H106" t="n">
+        <v>1300</v>
+      </c>
+      <c r="I106" t="n">
+        <v>850</v>
+      </c>
+      <c r="J106" t="n">
+        <v>10</v>
+      </c>
+      <c r="K106" t="n">
+        <v>2</v>
+      </c>
+      <c r="L106" t="n">
+        <v>26</v>
+      </c>
+      <c r="M106" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="N106" t="n">
+        <v>130000</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Huawei SUN2000-100KTL-M1</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>Ficha técnica oficial — sistema 1500V granja FV</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F107" t="n">
+        <v>200</v>
+      </c>
+      <c r="G107" t="n">
+        <v>200</v>
+      </c>
+      <c r="H107" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I107" t="n">
+        <v>780</v>
+      </c>
+      <c r="J107" t="n">
+        <v>12</v>
+      </c>
+      <c r="K107" t="n">
+        <v>2</v>
+      </c>
+      <c r="L107" t="n">
+        <v>26</v>
+      </c>
+      <c r="M107" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="N107" t="n">
+        <v>135000</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Sungrow SG110CX</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>Ficha técnica oficial — sistema 1500V granja FV</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F108" t="n">
+        <v>200</v>
+      </c>
+      <c r="G108" t="n">
+        <v>200</v>
+      </c>
+      <c r="H108" t="n">
+        <v>1500</v>
+      </c>
+      <c r="I108" t="n">
+        <v>850</v>
+      </c>
+      <c r="J108" t="n">
+        <v>12</v>
+      </c>
+      <c r="K108" t="n">
+        <v>2</v>
+      </c>
+      <c r="L108" t="n">
+        <v>26</v>
+      </c>
+      <c r="M108" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="N108" t="n">
+        <v>148500</v>
       </c>
     </row>
   </sheetData>
@@ -5721,6 +5862,26 @@
           <t>CATÁLOGO DE BATERÍAS — BIPV COLOMBIA  |  26 modelos  |  Alta tensión 300–870 V</t>
         </is>
       </c>
+      <c r="B1" s="6" t="n"/>
+      <c r="C1" s="6" t="n"/>
+      <c r="D1" s="6" t="n"/>
+      <c r="E1" s="6" t="n"/>
+      <c r="F1" s="6" t="n"/>
+      <c r="G1" s="6" t="n"/>
+      <c r="H1" s="6" t="n"/>
+      <c r="I1" s="6" t="n"/>
+      <c r="J1" s="6" t="n"/>
+      <c r="K1" s="6" t="n"/>
+      <c r="L1" s="6" t="n"/>
+      <c r="M1" s="6" t="n"/>
+      <c r="N1" s="6" t="n"/>
+      <c r="O1" s="6" t="n"/>
+      <c r="P1" s="6" t="n"/>
+      <c r="Q1" s="6" t="n"/>
+      <c r="R1" s="6" t="n"/>
+      <c r="S1" s="6" t="n"/>
+      <c r="T1" s="6" t="n"/>
+      <c r="U1" s="7" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
@@ -7613,6 +7774,25 @@
           <t>⚠ Pendiente para TODOS los modelos: DoD (%), Eficiencia RTE (%), Garantía (años), Temperatura operación, Costo (USD). Solicitar al proveedor para marcar 'Datos completos = Si'.</t>
         </is>
       </c>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="6" t="n"/>
+      <c r="K31" s="6" t="n"/>
+      <c r="L31" s="6" t="n"/>
+      <c r="M31" s="6" t="n"/>
+      <c r="N31" s="6" t="n"/>
+      <c r="O31" s="6" t="n"/>
+      <c r="P31" s="6" t="n"/>
+      <c r="Q31" s="6" t="n"/>
+      <c r="R31" s="6" t="n"/>
+      <c r="S31" s="6" t="n"/>
+      <c r="T31" s="6" t="n"/>
+      <c r="U31" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>

<commit_message>
Agrega el inversor real INVT MG750TL al catálogo (validación PVsyst CdTe)
Es el inversor con el que se corrió la última prueba real de PVsyst 8.1.5
(caso CdTe, ver DIAGNOSTICO_JRC_HULD_PRIMARIO_CDTE.md / DIAGNOSTICO_
RECOMBINACION_CDTE.md), pero no estaba en el catálogo de la app. Datos
verificados contra 2 fuentes reales: la ficha oficial INVT (rev. 2020.07)
y la pantalla real de PVsyst usada en esa corrida -- coinciden exacto en
tensión DC máxima (400V), potencia CA nominal (750W) y eficiencia máxima
(96,80%); la discrepancia real en la ventana MPPT entre ambas fuentes
queda documentada en el campo Notas, no oculta.

941/941 tests (2 nuevos).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gRCfBjq8vii432YfHyH35
</commit_message>
<xml_diff>
--- a/bipv_python/datos/inversores_catalogo.xlsx
+++ b/bipv_python/datos/inversores_catalogo.xlsx
@@ -643,7 +643,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W110"/>
+  <dimension ref="A1:W111"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col width="29.7109375" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -6205,6 +6205,60 @@
       </c>
       <c r="O110" t="n">
         <v>15</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Si</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>MG750TL</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>INVT-MG-0.75-6kW_datasheet_2020.07_V1.0.pdf + verificado contra pantalla real PVsyst 8.1.5</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>400</v>
+      </c>
+      <c r="F111" t="n">
+        <v>60</v>
+      </c>
+      <c r="G111" t="n">
+        <v>60</v>
+      </c>
+      <c r="H111" t="n">
+        <v>350</v>
+      </c>
+      <c r="I111" t="n">
+        <v>60</v>
+      </c>
+      <c r="J111" t="n">
+        <v>1</v>
+      </c>
+      <c r="K111" t="n">
+        <v>1</v>
+      </c>
+      <c r="N111" t="n">
+        <v>900</v>
+      </c>
+      <c r="O111" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P111" t="inlineStr">
+        <is>
+          <t>INVT Solar Technology</t>
+        </is>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>Eficiencia máxima 96,80% (idéntica en ficha oficial y pantalla PVsyst). Eficiencia Euro: 95,95% (ficha oficial) / 96,00% (PVsyst) -- diferencia menor, no resuelta. Corriente AC nominal ficha PVsyst: 3,26A (=750W/230V); corriente AC máxima ficha oficial: 3,6A (=~828W/230V, coherente con 'Potencia CA máxima 0,80kW' vista en PVsyst). Ventana MPPT de la ficha oficial 2020 es más amplia (50-400V) que la usada en la corrida real de PVsyst (60-350V) -- se usó esta última por ser la validada.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Corrige bug real: MG750TL no evaluaba compatibilidad en Dimensionamiento
Verificando el inversor recién agregado contra la config real ya validada
(ASP-ST1-T40, 3 en serie x 4 strings), evaluar_compatibilidad_string()
devolvía evaluable=False ("ficha incompleta") -- había dejado la corriente
máxima de entrada en blanco porque ninguna fuente la publicaba
directamente (PVsyst mostró "N/A"), pero ese campo es requerido por la
función, no opcional.

Corregido con un valor DERIVADO (no inventado) de 2 números ya reales:
900W (potencia DC máxima) / 60V (Vmppt mínimo) = 15A, el peor caso físico
de corriente a máxima potencia en el extremo inferior de la ventana MPPT.
Verificado: la config real ahora da compatible=True, ratio DC:AC=1.01 🟢.

942/942 tests (1 nuevo).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016gRCfBjq8vii432YfHyH35
</commit_message>
<xml_diff>
--- a/bipv_python/datos/inversores_catalogo.xlsx
+++ b/bipv_python/datos/inversores_catalogo.xlsx
@@ -6244,6 +6244,12 @@
       <c r="K111" t="n">
         <v>1</v>
       </c>
+      <c r="L111" t="n">
+        <v>15</v>
+      </c>
+      <c r="M111" t="n">
+        <v>15</v>
+      </c>
       <c r="N111" t="n">
         <v>900</v>
       </c>
@@ -6257,7 +6263,7 @@
       </c>
       <c r="W111" t="inlineStr">
         <is>
-          <t>Eficiencia máxima 96,80% (idéntica en ficha oficial y pantalla PVsyst). Eficiencia Euro: 95,95% (ficha oficial) / 96,00% (PVsyst) -- diferencia menor, no resuelta. Corriente AC nominal ficha PVsyst: 3,26A (=750W/230V); corriente AC máxima ficha oficial: 3,6A (=~828W/230V, coherente con 'Potencia CA máxima 0,80kW' vista en PVsyst). Ventana MPPT de la ficha oficial 2020 es más amplia (50-400V) que la usada en la corrida real de PVsyst (60-350V) -- se usó esta última por ser la validada.</t>
+          <t>Eficiencia máxima 96,80% (idéntica en ficha oficial y pantalla PVsyst). Eficiencia Euro: 95,95% (ficha oficial) / 96,00% (PVsyst) -- diferencia menor, no resuelta. Corriente AC nominal ficha PVsyst: 3,26A (=750W/230V); corriente AC máxima ficha oficial: 3,6A (=~828W/230V, coherente con 'Potencia CA máxima 0,80kW' vista en PVsyst). Ventana MPPT de la ficha oficial 2020 es más amplia (50-400V) que la usada en la corrida real de PVsyst (60-350V) -- se usó esta última por ser la validada. Corriente máxima de entrada (15A): DERIVADA de 900W/60V (potencia DC máxima real / Vmppt mínimo real), no publicada directamente por ninguna fuente -- sin este valor, evaluar_compatibilidad_string() no podía evaluar ninguna configuración con este inversor.</t>
         </is>
       </c>
     </row>

</xml_diff>